<commit_message>
Add 2m LPF values and resolve ERC findings
</commit_message>
<xml_diff>
--- a/Wsprry-Pi-LPF/LPF-(C-L-C)-and-DC-Blocking-Filters.xlsx
+++ b/Wsprry-Pi-LPF/LPF-(C-L-C)-and-DC-Blocking-Filters.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LPF" sheetId="1" r:id="Re163c847e5294024"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="2" r:id="Rfe554c0f3ece4504"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LPF" sheetId="1" r:id="Rc4f460b90e9c4746"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="2" r:id="Rfe5f3ecb69964f66"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -155,7 +155,7 @@
     <x:t xml:space="preserve">17.851000 MHz</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">60m</x:t>
+    <x:t xml:space="preserve">60 &amp; 80m</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">5,288.700 kHz +/- 100 Hz</x:t>
@@ -203,7 +203,7 @@
     <x:t xml:space="preserve">35.201000 MHz</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">30m</x:t>
+    <x:t xml:space="preserve">30 &amp; 40m</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">10,140.200 kHz +/- 100 Hz</x:t>
@@ -251,7 +251,7 @@
     <x:t xml:space="preserve">67.777500 MHz</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">20m</x:t>
+    <x:t xml:space="preserve">20 &amp; 22m</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">14,097.100 kHz +/- 100 Hz</x:t>
@@ -299,7 +299,7 @@
     <x:t xml:space="preserve">90.531000 MHz</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">15m</x:t>
+    <x:t xml:space="preserve">15 &amp; 17m</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">21,096.100 kHz +/- 100 Hz</x:t>
@@ -347,7 +347,7 @@
     <x:t xml:space="preserve">124.631000 MHz</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">10m</x:t>
+    <x:t xml:space="preserve">10 &amp; 12m</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">28,126.100 kHz +/- 100 Hz</x:t>
@@ -402,10 +402,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
+    <x:numFmt numFmtId="164" formatCode="0.000\ &quot;dB&quot;"/>
     <x:numFmt numFmtId="200" formatCode="0.000 &quot;dB&quot;"/>
   </x:numFmts>
-  <x:fonts count="10">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="12"/>
       <x:color theme="1"/>
@@ -415,10 +416,6 @@
       <x:b/>
       <x:sz val="12"/>
       <x:color theme="1"/>
-      <x:name val="Aptos Narrow"/>
-    </x:font>
-    <x:font>
-      <x:sz val="8"/>
       <x:name val="Aptos Narrow"/>
     </x:font>
     <x:font>
@@ -446,12 +443,7 @@
     </x:font>
     <x:font>
       <x:sz val="12"/>
-      <x:color theme="2" tint="-0.74999"/>
-      <x:name val="Aptos Narrow"/>
-    </x:font>
-    <x:font>
-      <x:sz val="12"/>
-      <x:color theme="2" tint="-0.74999"/>
+      <x:color theme="2" tint="-0.74996"/>
       <x:name val="Aptos Narrow"/>
     </x:font>
     <x:font>
@@ -460,7 +452,7 @@
       <x:name val="Aptos Narrow"/>
     </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -470,21 +462,6 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor theme="1"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFFF00"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFFFFF"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -503,7 +480,7 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="6">
+  <x:borders count="7">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -572,66 +549,86 @@
         <x:color indexed="64"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF000000"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FF000000"/>
+      </x:right>
+      <x:top style="double">
+        <x:color rgb="FF000000"/>
+      </x:top>
+      <x:bottom style="double">
+        <x:color rgb="FF000000"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="2">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="40">
+  <x:cellXfs count="48">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <x:xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <x:xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <x:xf numFmtId="164" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyFill="1"/>
-    <x:xf numFmtId="200" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="200" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
@@ -641,13 +638,35 @@
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="2">
     <x:cellStyle name="Hyperlink" xfId="1"/>
@@ -851,12 +870,12 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <x:cols>
-    <x:col min="1" max="1" width="6.1640625" customWidth="1"/>
-    <x:col min="2" max="2" width="6.6640625" customWidth="1"/>
-    <x:col min="3" max="3" width="22.33203125" customWidth="1"/>
-    <x:col min="4" max="4" width="24.1640625" customWidth="1"/>
-    <x:col min="5" max="5" width="15.83203125" customWidth="1"/>
-    <x:col min="6" max="9" width="14.6640625" customWidth="1"/>
+    <x:col min="1" max="2" width="8.6640625" customWidth="1"/>
+    <x:col min="3" max="3" width="22.5" customWidth="1"/>
+    <x:col min="4" max="4" width="24.33203125" customWidth="1"/>
+    <x:col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <x:col min="6" max="6" width="15.1640625" customWidth="1"/>
+    <x:col min="7" max="9" width="14.83203125" customWidth="1"/>
     <x:col min="10" max="10" width="13.6640625" customWidth="1"/>
     <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="14" hidden="0" customWidth="1"/>
@@ -953,214 +972,214 @@
       <x:c r="J2" s="4" t="str">
         <x:v>139.979 kHz</x:v>
       </x:c>
-      <x:c r="K2" s="19" t="n">
+      <x:c r="K2" s="24" t="n">
         <x:v>1.004</x:v>
       </x:c>
-      <x:c r="L2" s="32" t="str">
+      <x:c r="L2" s="30" t="str">
         <x:v>2.4 nF +
 47 nF</x:v>
       </x:c>
-      <x:c r="M2" s="32" t="str">
+      <x:c r="M2" s="30" t="str">
         <x:v>64.9 µH</x:v>
       </x:c>
-      <x:c r="N2" s="32" t="str">
+      <x:c r="N2" s="30" t="str">
         <x:v>9.1 nF +
 62 nF</x:v>
       </x:c>
-      <x:c r="O2" s="32" t="str">
+      <x:c r="O2" s="30" t="str">
         <x:v>68.1 µH</x:v>
       </x:c>
-      <x:c r="P2" s="32" t="str">
+      <x:c r="P2" s="30" t="str">
         <x:v>9.1 nF +
 62 nF</x:v>
       </x:c>
-      <x:c r="Q2" s="32" t="str">
+      <x:c r="Q2" s="30" t="str">
         <x:v>64.9 µH</x:v>
       </x:c>
-      <x:c r="R2" s="32" t="str">
+      <x:c r="R2" s="30" t="str">
         <x:v>2.4 nF +
 47 nF</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="6">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B3" s="7" t="s">
+      <x:c r="A3" s="5">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B3" s="6" t="s">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="C3" s="7" t="s">
+      <x:c r="C3" s="6" t="s">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="D3" s="7" t="s">
+      <x:c r="D3" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="E3" s="7" t="s">
+      <x:c r="E3" s="6" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="F3" s="7" t="s">
+      <x:c r="F3" s="6" t="s">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="G3" s="7" t="s">
+      <x:c r="G3" s="6" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="H3" s="7" t="s">
+      <x:c r="H3" s="6" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="I3" s="7" t="s">
+      <x:c r="I3" s="6" t="s">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="J3" s="7" t="str">
+      <x:c r="J3" s="6" t="str">
         <x:v>485.062 kHz</x:v>
       </x:c>
-      <x:c r="K3" s="20" t="n">
+      <x:c r="K3" s="25" t="n">
         <x:v>0.821</x:v>
       </x:c>
-      <x:c r="L3" s="33" t="str">
+      <x:c r="L3" s="31" t="str">
         <x:v>14.3 nF</x:v>
       </x:c>
-      <x:c r="M3" s="33" t="str">
+      <x:c r="M3" s="31" t="str">
         <x:v>18.7 µH</x:v>
       </x:c>
-      <x:c r="N3" s="33" t="str">
+      <x:c r="N3" s="31" t="str">
         <x:v>560 pF +
 20 nF</x:v>
       </x:c>
-      <x:c r="O3" s="33" t="str">
+      <x:c r="O3" s="31" t="str">
         <x:v>19.6 µH</x:v>
       </x:c>
-      <x:c r="P3" s="33" t="str">
+      <x:c r="P3" s="31" t="str">
         <x:v>560 pF +
 20 nF</x:v>
       </x:c>
-      <x:c r="Q3" s="33" t="str">
+      <x:c r="Q3" s="31" t="str">
         <x:v>18.7 µH</x:v>
       </x:c>
-      <x:c r="R3" s="33" t="str">
+      <x:c r="R3" s="31" t="str">
         <x:v>14.3 nF</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="9">
+      <x:c r="A4" s="7">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B4" s="10" t="s">
+      <x:c r="B4" s="8" t="s">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="C4" s="10" t="s">
+      <x:c r="C4" s="8" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="D4" s="10" t="s">
+      <x:c r="D4" s="8" t="s">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="E4" s="10" t="s">
+      <x:c r="E4" s="8" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="F4" s="10" t="s">
+      <x:c r="F4" s="8" t="s">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="G4" s="10" t="s">
+      <x:c r="G4" s="8" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="H4" s="10" t="s">
+      <x:c r="H4" s="8" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="I4" s="10" t="s">
+      <x:c r="I4" s="8" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="J4" s="10" t="str">
+      <x:c r="J4" s="8" t="str">
         <x:v>1.870865 MHz</x:v>
       </x:c>
-      <x:c r="K4" s="21" t="n">
+      <x:c r="K4" s="26" t="n">
         <x:v>0.953</x:v>
       </x:c>
-      <x:c r="L4" s="34" t="str">
+      <x:c r="L4" s="32" t="str">
         <x:v>100 pF +
 3.6 nF</x:v>
       </x:c>
-      <x:c r="M4" s="34" t="str">
+      <x:c r="M4" s="32" t="str">
         <x:v>4.87 µH</x:v>
       </x:c>
-      <x:c r="N4" s="34" t="str">
+      <x:c r="N4" s="32" t="str">
         <x:v>200 pF +
 5.1 nF</x:v>
       </x:c>
-      <x:c r="O4" s="34" t="str">
+      <x:c r="O4" s="32" t="str">
         <x:v>5.11 µH</x:v>
       </x:c>
-      <x:c r="P4" s="34" t="str">
+      <x:c r="P4" s="32" t="str">
         <x:v>200 pF +
 5.1 nF</x:v>
       </x:c>
-      <x:c r="Q4" s="34" t="str">
+      <x:c r="Q4" s="32" t="str">
         <x:v>4.87 µH</x:v>
       </x:c>
-      <x:c r="R4" s="34" t="str">
+      <x:c r="R4" s="32" t="str">
         <x:v>100 pF +
 3.6 nF</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="28" hidden="1" customHeight="1">
-      <x:c r="A5" s="15">
+      <x:c r="A5" s="21">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B5" s="13" t="s">
+      <x:c r="B5" s="9" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="C5" s="13" t="s">
+      <x:c r="C5" s="9" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="D5" s="13" t="s">
+      <x:c r="D5" s="9" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="E5" s="13" t="s">
+      <x:c r="E5" s="9" t="s">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="F5" s="13" t="s">
+      <x:c r="F5" s="9" t="s">
         <x:v>44</x:v>
       </x:c>
-      <x:c r="G5" s="13" t="s">
+      <x:c r="G5" s="9" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="H5" s="13" t="s">
+      <x:c r="H5" s="9" t="s">
         <x:v>46</x:v>
       </x:c>
-      <x:c r="I5" s="13" t="s">
+      <x:c r="I5" s="9" t="s">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="J5" s="13" t="str">
+      <x:c r="J5" s="9" t="str">
         <x:v>3.639086 MHz</x:v>
       </x:c>
-      <x:c r="K5" s="22" t="n">
+      <x:c r="K5" s="27" t="n">
         <x:v>0.83</x:v>
       </x:c>
-      <x:c r="L5" s="35" t="str">
+      <x:c r="L5" s="33" t="str">
         <x:v>1.91 nF</x:v>
       </x:c>
-      <x:c r="M5" s="35" t="str">
+      <x:c r="M5" s="33" t="str">
         <x:v>2.49 µH</x:v>
       </x:c>
-      <x:c r="N5" s="35" t="str">
+      <x:c r="N5" s="33" t="str">
         <x:v>43 pF +
 2.7 nF</x:v>
       </x:c>
-      <x:c r="O5" s="35" t="str">
+      <x:c r="O5" s="33" t="str">
         <x:v>2.61 µH</x:v>
       </x:c>
-      <x:c r="P5" s="35" t="str">
+      <x:c r="P5" s="33" t="str">
         <x:v>43 pF +
 2.7 nF</x:v>
       </x:c>
-      <x:c r="Q5" s="35" t="str">
+      <x:c r="Q5" s="33" t="str">
         <x:v>2.49 µH</x:v>
       </x:c>
-      <x:c r="R5" s="35" t="str">
+      <x:c r="R5" s="33" t="str">
         <x:v>1.91 nF</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="28" customHeight="1">
-      <x:c r="A6" s="16"/>
-      <x:c r="B6" s="4" t="s">
+      <x:c r="A6" s="22"/>
+      <x:c r="B6" s="23" t="s">
         <x:v>48</x:v>
       </x:c>
       <x:c r="C6" s="4" t="s">
@@ -1187,98 +1206,98 @@
       <x:c r="J6" s="4" t="str">
         <x:v>5.380206 MHz</x:v>
       </x:c>
-      <x:c r="K6" s="23" t="n">
+      <x:c r="K6" s="28" t="n">
         <x:v>0.994</x:v>
       </x:c>
-      <x:c r="L6" s="32" t="str">
+      <x:c r="L6" s="30" t="str">
         <x:v>470 pF +
 820 pF</x:v>
       </x:c>
-      <x:c r="M6" s="32" t="str">
+      <x:c r="M6" s="30" t="str">
         <x:v>1.69 µH</x:v>
       </x:c>
-      <x:c r="N6" s="32" t="str">
+      <x:c r="N6" s="30" t="str">
         <x:v>43 pF +
 1.8 nF</x:v>
       </x:c>
-      <x:c r="O6" s="32" t="str">
+      <x:c r="O6" s="30" t="str">
         <x:v>1.78 µH</x:v>
       </x:c>
-      <x:c r="P6" s="32" t="str">
+      <x:c r="P6" s="30" t="str">
         <x:v>43 pF +
 1.8 nF</x:v>
       </x:c>
-      <x:c r="Q6" s="32" t="str">
+      <x:c r="Q6" s="30" t="str">
         <x:v>1.69 µH</x:v>
       </x:c>
-      <x:c r="R6" s="32" t="str">
+      <x:c r="R6" s="30" t="str">
         <x:v>470 pF +
 820 pF</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="28" hidden="1" customHeight="1">
-      <x:c r="A7" s="15">
+      <x:c r="A7" s="21">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B7" s="13" t="s">
+      <x:c r="B7" s="9" t="s">
         <x:v>56</x:v>
       </x:c>
-      <x:c r="C7" s="13" t="s">
+      <x:c r="C7" s="9" t="s">
         <x:v>57</x:v>
       </x:c>
-      <x:c r="D7" s="13" t="s">
+      <x:c r="D7" s="9" t="s">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="E7" s="13" t="s">
+      <x:c r="E7" s="9" t="s">
         <x:v>59</x:v>
       </x:c>
-      <x:c r="F7" s="13" t="s">
+      <x:c r="F7" s="9" t="s">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="G7" s="13" t="s">
+      <x:c r="G7" s="9" t="s">
         <x:v>61</x:v>
       </x:c>
-      <x:c r="H7" s="13" t="s">
+      <x:c r="H7" s="9" t="s">
         <x:v>62</x:v>
       </x:c>
-      <x:c r="I7" s="13" t="s">
+      <x:c r="I7" s="9" t="s">
         <x:v>63</x:v>
       </x:c>
-      <x:c r="J7" s="13" t="str">
+      <x:c r="J7" s="9" t="str">
         <x:v>7.157261 MHz</x:v>
       </x:c>
-      <x:c r="K7" s="22" t="n">
+      <x:c r="K7" s="27" t="n">
         <x:v>1.059</x:v>
       </x:c>
-      <x:c r="L7" s="35" t="str">
+      <x:c r="L7" s="33" t="str">
         <x:v>51 pF +
 910 pF</x:v>
       </x:c>
-      <x:c r="M7" s="35" t="str">
+      <x:c r="M7" s="33" t="str">
         <x:v>1.27 µH</x:v>
       </x:c>
-      <x:c r="N7" s="35" t="str">
+      <x:c r="N7" s="33" t="str">
         <x:v>110 pF +
 1.3 nF</x:v>
       </x:c>
-      <x:c r="O7" s="35" t="str">
+      <x:c r="O7" s="33" t="str">
         <x:v>1.3 µH</x:v>
       </x:c>
-      <x:c r="P7" s="35" t="str">
+      <x:c r="P7" s="33" t="str">
         <x:v>110 pF +
 1.3 nF</x:v>
       </x:c>
-      <x:c r="Q7" s="35" t="str">
+      <x:c r="Q7" s="33" t="str">
         <x:v>1.27 µH</x:v>
       </x:c>
-      <x:c r="R7" s="35" t="str">
+      <x:c r="R7" s="33" t="str">
         <x:v>51 pF +
 910 pF</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="28" customHeight="1">
-      <x:c r="A8" s="16"/>
-      <x:c r="B8" s="4" t="s">
+      <x:c r="A8" s="22"/>
+      <x:c r="B8" s="23" t="s">
         <x:v>64</x:v>
       </x:c>
       <x:c r="C8" s="4" t="s">
@@ -1305,90 +1324,90 @@
       <x:c r="J8" s="4" t="str">
         <x:v>10.343753 MHz</x:v>
       </x:c>
-      <x:c r="K8" s="23" t="n">
+      <x:c r="K8" s="28" t="n">
         <x:v>0.758</x:v>
       </x:c>
-      <x:c r="L8" s="32" t="str">
+      <x:c r="L8" s="30" t="str">
         <x:v>681 pF</x:v>
       </x:c>
-      <x:c r="M8" s="32" t="str">
+      <x:c r="M8" s="30" t="str">
         <x:v>866 nH</x:v>
       </x:c>
-      <x:c r="N8" s="32" t="str">
+      <x:c r="N8" s="30" t="str">
         <x:v>976 pF</x:v>
       </x:c>
-      <x:c r="O8" s="32" t="str">
+      <x:c r="O8" s="30" t="str">
         <x:v>909 nH</x:v>
       </x:c>
-      <x:c r="P8" s="32" t="str">
+      <x:c r="P8" s="30" t="str">
         <x:v>976 pF</x:v>
       </x:c>
-      <x:c r="Q8" s="32" t="str">
+      <x:c r="Q8" s="30" t="str">
         <x:v>866 nH</x:v>
       </x:c>
-      <x:c r="R8" s="32" t="str">
+      <x:c r="R8" s="30" t="str">
         <x:v>681 pF</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="28" hidden="1" customHeight="1">
-      <x:c r="A9" s="15">
+      <x:c r="A9" s="21">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B9" s="13" t="s">
+      <x:c r="B9" s="9" t="s">
         <x:v>72</x:v>
       </x:c>
-      <x:c r="C9" s="13" t="s">
+      <x:c r="C9" s="9" t="s">
         <x:v>73</x:v>
       </x:c>
-      <x:c r="D9" s="13" t="s">
+      <x:c r="D9" s="9" t="s">
         <x:v>74</x:v>
       </x:c>
-      <x:c r="E9" s="13" t="s">
+      <x:c r="E9" s="9" t="s">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="F9" s="13" t="s">
+      <x:c r="F9" s="9" t="s">
         <x:v>76</x:v>
       </x:c>
-      <x:c r="G9" s="13" t="s">
+      <x:c r="G9" s="9" t="s">
         <x:v>77</x:v>
       </x:c>
-      <x:c r="H9" s="13" t="s">
+      <x:c r="H9" s="9" t="s">
         <x:v>78</x:v>
       </x:c>
-      <x:c r="I9" s="13" t="s">
+      <x:c r="I9" s="9" t="s">
         <x:v>79</x:v>
       </x:c>
-      <x:c r="J9" s="13" t="str">
+      <x:c r="J9" s="9" t="str">
         <x:v>13.797760 MHz</x:v>
       </x:c>
-      <x:c r="K9" s="22" t="n">
+      <x:c r="K9" s="27" t="n">
         <x:v>0.928</x:v>
       </x:c>
-      <x:c r="L9" s="35" t="str">
+      <x:c r="L9" s="33" t="str">
         <x:v>511 pF</x:v>
       </x:c>
-      <x:c r="M9" s="35" t="str">
+      <x:c r="M9" s="33" t="str">
         <x:v>649 nH</x:v>
       </x:c>
-      <x:c r="N9" s="35" t="str">
+      <x:c r="N9" s="33" t="str">
         <x:v>732 pF</x:v>
       </x:c>
-      <x:c r="O9" s="35" t="str">
+      <x:c r="O9" s="33" t="str">
         <x:v>681 nH</x:v>
       </x:c>
-      <x:c r="P9" s="35" t="str">
+      <x:c r="P9" s="33" t="str">
         <x:v>732 pF</x:v>
       </x:c>
-      <x:c r="Q9" s="35" t="str">
+      <x:c r="Q9" s="33" t="str">
         <x:v>649 nH</x:v>
       </x:c>
-      <x:c r="R9" s="35" t="str">
+      <x:c r="R9" s="33" t="str">
         <x:v>511 pF</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="28" customHeight="1">
-      <x:c r="A10" s="16"/>
-      <x:c r="B10" s="4" t="s">
+      <x:c r="A10" s="22"/>
+      <x:c r="B10" s="23" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="C10" s="4" t="s">
@@ -1415,98 +1434,98 @@
       <x:c r="J10" s="4" t="str">
         <x:v>14.343209 MHz</x:v>
       </x:c>
-      <x:c r="K10" s="23" t="n">
+      <x:c r="K10" s="28" t="n">
         <x:v>0.982</x:v>
       </x:c>
-      <x:c r="L10" s="32" t="str">
+      <x:c r="L10" s="30" t="str">
         <x:v>13 pF +
 470 pF</x:v>
       </x:c>
-      <x:c r="M10" s="32" t="str">
+      <x:c r="M10" s="30" t="str">
         <x:v>634 nH</x:v>
       </x:c>
-      <x:c r="N10" s="32" t="str">
+      <x:c r="N10" s="30" t="str">
         <x:v>13 pF +
 680 pF</x:v>
       </x:c>
-      <x:c r="O10" s="32" t="str">
+      <x:c r="O10" s="30" t="str">
         <x:v>665 nH</x:v>
       </x:c>
-      <x:c r="P10" s="32" t="str">
+      <x:c r="P10" s="30" t="str">
         <x:v>13 pF +
 680 pF</x:v>
       </x:c>
-      <x:c r="Q10" s="32" t="str">
+      <x:c r="Q10" s="30" t="str">
         <x:v>634 nH</x:v>
       </x:c>
-      <x:c r="R10" s="32" t="str">
+      <x:c r="R10" s="30" t="str">
         <x:v>13 pF +
 470 pF</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="28" hidden="1" customHeight="1">
-      <x:c r="A11" s="15">
+      <x:c r="A11" s="21">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B11" s="13" t="s">
+      <x:c r="B11" s="9" t="s">
         <x:v>88</x:v>
       </x:c>
-      <x:c r="C11" s="13" t="s">
+      <x:c r="C11" s="9" t="s">
         <x:v>89</x:v>
       </x:c>
-      <x:c r="D11" s="13" t="s">
+      <x:c r="D11" s="9" t="s">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="E11" s="13" t="s">
+      <x:c r="E11" s="9" t="s">
         <x:v>91</x:v>
       </x:c>
-      <x:c r="F11" s="13" t="s">
+      <x:c r="F11" s="9" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="G11" s="13" t="s">
+      <x:c r="G11" s="9" t="s">
         <x:v>93</x:v>
       </x:c>
-      <x:c r="H11" s="13" t="s">
+      <x:c r="H11" s="9" t="s">
         <x:v>94</x:v>
       </x:c>
-      <x:c r="I11" s="13" t="s">
+      <x:c r="I11" s="9" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="J11" s="13" t="str">
+      <x:c r="J11" s="9" t="str">
         <x:v>18.458976 MHz</x:v>
       </x:c>
-      <x:c r="K11" s="22" t="n">
+      <x:c r="K11" s="27" t="n">
         <x:v>0.806</x:v>
       </x:c>
-      <x:c r="L11" s="35" t="str">
+      <x:c r="L11" s="33" t="str">
         <x:v>20 pF +
 360 pF</x:v>
       </x:c>
-      <x:c r="M11" s="35" t="str">
+      <x:c r="M11" s="33" t="str">
         <x:v>487 nH</x:v>
       </x:c>
-      <x:c r="N11" s="35" t="str">
+      <x:c r="N11" s="33" t="str">
         <x:v>75 pF +
 470 pF</x:v>
       </x:c>
-      <x:c r="O11" s="35" t="str">
+      <x:c r="O11" s="33" t="str">
         <x:v>511 nH</x:v>
       </x:c>
-      <x:c r="P11" s="35" t="str">
+      <x:c r="P11" s="33" t="str">
         <x:v>75 pF +
 470 pF</x:v>
       </x:c>
-      <x:c r="Q11" s="35" t="str">
+      <x:c r="Q11" s="33" t="str">
         <x:v>487 nH</x:v>
       </x:c>
-      <x:c r="R11" s="35" t="str">
+      <x:c r="R11" s="33" t="str">
         <x:v>20 pF +
 360 pF</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="28" customHeight="1">
-      <x:c r="A12" s="16"/>
-      <x:c r="B12" s="4" t="s">
+      <x:c r="A12" s="22"/>
+      <x:c r="B12" s="23" t="s">
         <x:v>96</x:v>
       </x:c>
       <x:c r="C12" s="4" t="s">
@@ -1533,96 +1552,96 @@
       <x:c r="J12" s="4" t="str">
         <x:v>21.472511 MHz</x:v>
       </x:c>
-      <x:c r="K12" s="23" t="n">
+      <x:c r="K12" s="28" t="n">
         <x:v>0.944</x:v>
       </x:c>
-      <x:c r="L12" s="32" t="str">
+      <x:c r="L12" s="30" t="str">
         <x:v>324 pF</x:v>
       </x:c>
-      <x:c r="M12" s="32" t="str">
+      <x:c r="M12" s="30" t="str">
         <x:v>422 nH</x:v>
       </x:c>
-      <x:c r="N12" s="32" t="str">
+      <x:c r="N12" s="30" t="str">
         <x:v>75 pF +
 390 pF</x:v>
       </x:c>
-      <x:c r="O12" s="32" t="str">
+      <x:c r="O12" s="30" t="str">
         <x:v>442 nH</x:v>
       </x:c>
-      <x:c r="P12" s="32" t="str">
+      <x:c r="P12" s="30" t="str">
         <x:v>75 pF +
 390 pF</x:v>
       </x:c>
-      <x:c r="Q12" s="32" t="str">
+      <x:c r="Q12" s="30" t="str">
         <x:v>422 nH</x:v>
       </x:c>
-      <x:c r="R12" s="32" t="str">
+      <x:c r="R12" s="30" t="str">
         <x:v>324 pF</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="28" hidden="1" customHeight="1">
-      <x:c r="A13" s="15">
+      <x:c r="A13" s="21">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B13" s="13" t="s">
+      <x:c r="B13" s="9" t="s">
         <x:v>104</x:v>
       </x:c>
-      <x:c r="C13" s="13" t="s">
+      <x:c r="C13" s="9" t="s">
         <x:v>105</x:v>
       </x:c>
-      <x:c r="D13" s="13" t="s">
+      <x:c r="D13" s="9" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="E13" s="13" t="s">
+      <x:c r="E13" s="9" t="s">
         <x:v>107</x:v>
       </x:c>
-      <x:c r="F13" s="13" t="s">
+      <x:c r="F13" s="9" t="s">
         <x:v>108</x:v>
       </x:c>
-      <x:c r="G13" s="13" t="s">
+      <x:c r="G13" s="9" t="s">
         <x:v>109</x:v>
       </x:c>
-      <x:c r="H13" s="13" t="s">
+      <x:c r="H13" s="9" t="s">
         <x:v>110</x:v>
       </x:c>
-      <x:c r="I13" s="13" t="s">
+      <x:c r="I13" s="9" t="s">
         <x:v>111</x:v>
       </x:c>
-      <x:c r="J13" s="13" t="str">
+      <x:c r="J13" s="9" t="str">
         <x:v>25.354603 MHz</x:v>
       </x:c>
-      <x:c r="K13" s="22" t="n">
+      <x:c r="K13" s="27" t="n">
         <x:v>1.002</x:v>
       </x:c>
-      <x:c r="L13" s="35" t="str">
+      <x:c r="L13" s="33" t="str">
         <x:v>4.3 pF +
 270 pF</x:v>
       </x:c>
-      <x:c r="M13" s="35" t="str">
+      <x:c r="M13" s="33" t="str">
         <x:v>357 nH</x:v>
       </x:c>
-      <x:c r="N13" s="35" t="str">
+      <x:c r="N13" s="33" t="str">
         <x:v>4.3 pF +
 390 pF</x:v>
       </x:c>
-      <x:c r="O13" s="35" t="str">
+      <x:c r="O13" s="33" t="str">
         <x:v>374 nH</x:v>
       </x:c>
-      <x:c r="P13" s="35" t="str">
+      <x:c r="P13" s="33" t="str">
         <x:v>4.3 pF +
 390 pF</x:v>
       </x:c>
-      <x:c r="Q13" s="35" t="str">
+      <x:c r="Q13" s="33" t="str">
         <x:v>357 nH</x:v>
       </x:c>
-      <x:c r="R13" s="35" t="str">
+      <x:c r="R13" s="33" t="str">
         <x:v>4.3 pF +
 270 pF</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="28" customHeight="1">
-      <x:c r="A14" s="16"/>
-      <x:c r="B14" s="4" t="s">
+      <x:c r="A14" s="22"/>
+      <x:c r="B14" s="23" t="s">
         <x:v>112</x:v>
       </x:c>
       <x:c r="C14" s="4" t="s">
@@ -1649,92 +1668,151 @@
       <x:c r="J14" s="4" t="str">
         <x:v>28.658718 MHz</x:v>
       </x:c>
-      <x:c r="K14" s="23" t="n">
+      <x:c r="K14" s="28" t="n">
         <x:v>0.855</x:v>
       </x:c>
-      <x:c r="L14" s="32" t="str">
+      <x:c r="L14" s="30" t="str">
         <x:v>243 pF</x:v>
       </x:c>
-      <x:c r="M14" s="32" t="str">
+      <x:c r="M14" s="30" t="str">
         <x:v>316 nH</x:v>
       </x:c>
-      <x:c r="N14" s="32" t="str">
+      <x:c r="N14" s="30" t="str">
         <x:v>348 pF</x:v>
       </x:c>
-      <x:c r="O14" s="32" t="str">
+      <x:c r="O14" s="30" t="str">
         <x:v>332 nH</x:v>
       </x:c>
-      <x:c r="P14" s="32" t="str">
+      <x:c r="P14" s="30" t="str">
         <x:v>348 pF</x:v>
       </x:c>
-      <x:c r="Q14" s="32" t="str">
+      <x:c r="Q14" s="30" t="str">
         <x:v>316 nH</x:v>
       </x:c>
-      <x:c r="R14" s="32" t="str">
+      <x:c r="R14" s="30" t="str">
         <x:v>243 pF</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="28" customHeight="1">
-      <x:c r="A15" s="9">
+      <x:c r="A15" s="7">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="B15" s="10" t="s">
+      <x:c r="B15" s="8" t="s">
         <x:v>118</x:v>
       </x:c>
-      <x:c r="C15" s="10" t="s">
+      <x:c r="C15" s="8" t="s">
         <x:v>119</x:v>
       </x:c>
-      <x:c r="D15" s="10" t="s">
+      <x:c r="D15" s="8" t="s">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="E15" s="10" t="s">
+      <x:c r="E15" s="8" t="s">
         <x:v>121</x:v>
       </x:c>
-      <x:c r="F15" s="10" t="s">
+      <x:c r="F15" s="8" t="s">
         <x:v>122</x:v>
       </x:c>
-      <x:c r="G15" s="10" t="s">
+      <x:c r="G15" s="8" t="s">
         <x:v>123</x:v>
       </x:c>
-      <x:c r="H15" s="10" t="s">
+      <x:c r="H15" s="8" t="s">
         <x:v>124</x:v>
       </x:c>
-      <x:c r="I15" s="10" t="s">
+      <x:c r="I15" s="8" t="s">
         <x:v>125</x:v>
       </x:c>
-      <x:c r="J15" s="10" t="str">
+      <x:c r="J15" s="8" t="str">
         <x:v>51.254605 MHz</x:v>
       </x:c>
-      <x:c r="K15" s="21" t="n">
+      <x:c r="K15" s="26" t="n">
         <x:v>0.844</x:v>
       </x:c>
-      <x:c r="L15" s="34" t="str">
+      <x:c r="L15" s="32" t="str">
         <x:v>5.1 pF +
 130 pF</x:v>
       </x:c>
-      <x:c r="M15" s="34" t="str">
+      <x:c r="M15" s="32" t="str">
         <x:v>178 nH</x:v>
       </x:c>
-      <x:c r="N15" s="34" t="str">
+      <x:c r="N15" s="32" t="str">
         <x:v>13 pF +
 180 pF</x:v>
       </x:c>
-      <x:c r="O15" s="34" t="str">
+      <x:c r="O15" s="32" t="str">
         <x:v>187 nH</x:v>
       </x:c>
-      <x:c r="P15" s="34" t="str">
+      <x:c r="P15" s="32" t="str">
         <x:v>13 pF +
 180 pF</x:v>
       </x:c>
-      <x:c r="Q15" s="34" t="str">
+      <x:c r="Q15" s="32" t="str">
         <x:v>178 nH</x:v>
       </x:c>
-      <x:c r="R15" s="34" t="str">
+      <x:c r="R15" s="32" t="str">
         <x:v>5.1 pF +
 130 pF</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="17"/>
+    <x:row r="16" ht="28" customHeight="1">
+      <x:c r="A16" s="41" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B16" s="42" t="str">
+        <x:v>2m</x:v>
+      </x:c>
+      <x:c r="C16" s="42" t="str">
+        <x:v>144,490.000 kHz +/- 100 Hz</x:v>
+      </x:c>
+      <x:c r="D16" s="42"/>
+      <x:c r="E16" s="42" t="str">
+        <x:v>144.490100 MHz</x:v>
+      </x:c>
+      <x:c r="F16" s="42" t="str">
+        <x:v>288.980200 MHz</x:v>
+      </x:c>
+      <x:c r="G16" s="42" t="str">
+        <x:v>433.470300 MHz</x:v>
+      </x:c>
+      <x:c r="H16" s="42" t="str">
+        <x:v>577.960400 MHz</x:v>
+      </x:c>
+      <x:c r="I16" s="42" t="str">
+        <x:v>722.450500 MHz</x:v>
+      </x:c>
+      <x:c r="J16" s="42" t="str">
+        <x:v>148.279504 MHz</x:v>
+      </x:c>
+      <x:c r="K16" s="45" t="n">
+        <x:v>0.376</x:v>
+      </x:c>
+      <x:c r="L16" s="44" t="str">
+        <x:v>47.5 pF</x:v>
+      </x:c>
+      <x:c r="M16" s="44" t="str">
+        <x:v>60.4 nH</x:v>
+      </x:c>
+      <x:c r="N16" s="44" t="str">
+        <x:v>68.1 pF</x:v>
+      </x:c>
+      <x:c r="O16" s="44" t="str">
+        <x:v>63.4 nH</x:v>
+      </x:c>
+      <x:c r="P16" s="44" t="str">
+        <x:v>68.1 pF</x:v>
+      </x:c>
+      <x:c r="Q16" s="44" t="str">
+        <x:v>60.4 nH</x:v>
+      </x:c>
+      <x:c r="R16" s="44" t="str">
+        <x:v>47.5 pF</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>2m WSPR source: https://www.wsprnet.org/drupal/sites/wsprnet.org/files/wspr-qrg.pdf</x:v>
+      </x:c>
+      <x:c r="B18"/>
+    </x:row>
     <x:row r="27">
       <x:c r="E27" s="1"/>
       <x:c r="F27" s="1"/>
@@ -1753,9 +1831,9 @@
     <x:mergeCell ref="A13:A14"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="R134e41ddec83417f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="R2dc0f0f46f1f41bc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="R57e4416a5bfa471a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="R97e800805bd54d65"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="R38694f4395e14740"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="R17929b620e924774"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1766,9 +1844,9 @@
   <x:sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <x:cols>
     <x:col min="1" max="1" width="7.110000133514404" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="7.21999979019165" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="8.220000267028809" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="7.21999979019165" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="7.21999979019165" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -1786,689 +1864,725 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="38" t="str">
+      <x:c r="A2" s="46" t="str">
+        <x:v>60.4 nH</x:v>
+      </x:c>
+      <x:c r="B2" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C2" s="46"/>
+      <x:c r="D2" s="47" t="str">
+        <x:v>4.3 pF</x:v>
+      </x:c>
+      <x:c r="E2" s="46" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F2" s="46"/>
+      <x:c r="G2" s="46"/>
+      <x:c r="H2" s="46"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="46" t="str">
+        <x:v>63.4 nH</x:v>
+      </x:c>
+      <x:c r="B3" s="46" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C3" s="46"/>
+      <x:c r="D3" s="47" t="str">
+        <x:v>5.1 pF</x:v>
+      </x:c>
+      <x:c r="E3" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F3" s="46"/>
+      <x:c r="G3" s="46"/>
+      <x:c r="H3" s="46"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="46" t="str">
         <x:v>178 nH</x:v>
       </x:c>
-      <x:c r="B2" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C2" s="38"/>
-      <x:c r="D2" s="39" t="str">
-        <x:v>4.3 pF</x:v>
-      </x:c>
-      <x:c r="E2" s="38" t="n">
+      <x:c r="B4" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C4" s="46"/>
+      <x:c r="D4" s="47" t="str">
+        <x:v>13 pF</x:v>
+      </x:c>
+      <x:c r="E4" s="46" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F4" s="46"/>
+      <x:c r="G4" s="46"/>
+      <x:c r="H4" s="46"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="46" t="str">
+        <x:v>187 nH</x:v>
+      </x:c>
+      <x:c r="B5" s="46" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C5" s="46"/>
+      <x:c r="D5" s="47" t="str">
+        <x:v>20 pF</x:v>
+      </x:c>
+      <x:c r="E5" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F5" s="46"/>
+      <x:c r="G5" s="46"/>
+      <x:c r="H5" s="46"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="46" t="str">
+        <x:v>316 nH</x:v>
+      </x:c>
+      <x:c r="B6" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C6" s="46"/>
+      <x:c r="D6" s="47" t="str">
+        <x:v>43 pF</x:v>
+      </x:c>
+      <x:c r="E6" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="F2" s="38"/>
-      <x:c r="G2" s="38"/>
-      <x:c r="H2" s="38"/>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="38" t="str">
-        <x:v>187 nH</x:v>
-      </x:c>
-      <x:c r="B3" s="38" t="n">
+      <x:c r="F6" s="46"/>
+      <x:c r="G6" s="46"/>
+      <x:c r="H6" s="46"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="46" t="str">
+        <x:v>332 nH</x:v>
+      </x:c>
+      <x:c r="B7" s="46" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C3" s="38"/>
-      <x:c r="D3" s="39" t="str">
-        <x:v>5.1 pF</x:v>
-      </x:c>
-      <x:c r="E3" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F3" s="38"/>
-      <x:c r="G3" s="38"/>
-      <x:c r="H3" s="38"/>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="38" t="str">
-        <x:v>316 nH</x:v>
-      </x:c>
-      <x:c r="B4" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C4" s="38"/>
-      <x:c r="D4" s="39" t="str">
-        <x:v>13 pF</x:v>
-      </x:c>
-      <x:c r="E4" s="38" t="n">
+      <x:c r="C7" s="46"/>
+      <x:c r="D7" s="47" t="str">
+        <x:v>47.5 pF</x:v>
+      </x:c>
+      <x:c r="E7" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F7" s="46"/>
+      <x:c r="G7" s="46"/>
+      <x:c r="H7" s="46"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="46" t="str">
+        <x:v>357 nH</x:v>
+      </x:c>
+      <x:c r="B8" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C8" s="46"/>
+      <x:c r="D8" s="47" t="str">
+        <x:v>51 pF</x:v>
+      </x:c>
+      <x:c r="E8" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F8" s="46"/>
+      <x:c r="G8" s="46"/>
+      <x:c r="H8" s="46"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="46" t="str">
+        <x:v>374 nH</x:v>
+      </x:c>
+      <x:c r="B9" s="46" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C9" s="46"/>
+      <x:c r="D9" s="47" t="str">
+        <x:v>68.1 pF</x:v>
+      </x:c>
+      <x:c r="E9" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F9" s="46"/>
+      <x:c r="G9" s="46"/>
+      <x:c r="H9" s="46"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="46" t="str">
+        <x:v>422 nH</x:v>
+      </x:c>
+      <x:c r="B10" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C10" s="46"/>
+      <x:c r="D10" s="47" t="str">
+        <x:v>75 pF</x:v>
+      </x:c>
+      <x:c r="E10" s="46" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F10" s="46"/>
+      <x:c r="G10" s="46"/>
+      <x:c r="H10" s="46"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="46" t="str">
+        <x:v>442 nH</x:v>
+      </x:c>
+      <x:c r="B11" s="46" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C11" s="46"/>
+      <x:c r="D11" s="47" t="str">
+        <x:v>100 pF</x:v>
+      </x:c>
+      <x:c r="E11" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F11" s="46"/>
+      <x:c r="G11" s="46"/>
+      <x:c r="H11" s="46"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="46" t="str">
+        <x:v>487 nH</x:v>
+      </x:c>
+      <x:c r="B12" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C12" s="46"/>
+      <x:c r="D12" s="47" t="str">
+        <x:v>110 pF</x:v>
+      </x:c>
+      <x:c r="E12" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F12" s="46"/>
+      <x:c r="G12" s="46"/>
+      <x:c r="H12" s="46"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="46" t="str">
+        <x:v>511 nH</x:v>
+      </x:c>
+      <x:c r="B13" s="46" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C13" s="46"/>
+      <x:c r="D13" s="47" t="str">
+        <x:v>130 pF</x:v>
+      </x:c>
+      <x:c r="E13" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F13" s="46"/>
+      <x:c r="G13" s="46"/>
+      <x:c r="H13" s="46"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="46" t="str">
+        <x:v>634 nH</x:v>
+      </x:c>
+      <x:c r="B14" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C14" s="46"/>
+      <x:c r="D14" s="47" t="str">
+        <x:v>180 pF</x:v>
+      </x:c>
+      <x:c r="E14" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F14" s="46"/>
+      <x:c r="G14" s="46"/>
+      <x:c r="H14" s="46"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="46" t="str">
+        <x:v>649 nH</x:v>
+      </x:c>
+      <x:c r="B15" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C15" s="46"/>
+      <x:c r="D15" s="47" t="str">
+        <x:v>200 pF</x:v>
+      </x:c>
+      <x:c r="E15" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F15" s="46"/>
+      <x:c r="G15" s="46"/>
+      <x:c r="H15" s="46"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="46" t="str">
+        <x:v>665 nH</x:v>
+      </x:c>
+      <x:c r="B16" s="46" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C16" s="46"/>
+      <x:c r="D16" s="47" t="str">
+        <x:v>243 pF</x:v>
+      </x:c>
+      <x:c r="E16" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F16" s="46"/>
+      <x:c r="G16" s="46"/>
+      <x:c r="H16" s="46"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="46" t="str">
+        <x:v>681 nH</x:v>
+      </x:c>
+      <x:c r="B17" s="46" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C17" s="46"/>
+      <x:c r="D17" s="47" t="str">
+        <x:v>270 pF</x:v>
+      </x:c>
+      <x:c r="E17" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F17" s="46"/>
+      <x:c r="G17" s="46"/>
+      <x:c r="H17" s="46"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="46" t="str">
+        <x:v>866 nH</x:v>
+      </x:c>
+      <x:c r="B18" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C18" s="46"/>
+      <x:c r="D18" s="47" t="str">
+        <x:v>324 pF</x:v>
+      </x:c>
+      <x:c r="E18" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F18" s="46"/>
+      <x:c r="G18" s="46"/>
+      <x:c r="H18" s="46"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="46" t="str">
+        <x:v>909 nH</x:v>
+      </x:c>
+      <x:c r="B19" s="46" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C19" s="46"/>
+      <x:c r="D19" s="47" t="str">
+        <x:v>348 pF</x:v>
+      </x:c>
+      <x:c r="E19" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F19" s="46"/>
+      <x:c r="G19" s="46"/>
+      <x:c r="H19" s="46"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="46" t="str">
+        <x:v>1.27 µH</x:v>
+      </x:c>
+      <x:c r="B20" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C20" s="46"/>
+      <x:c r="D20" s="47" t="str">
+        <x:v>360 pF</x:v>
+      </x:c>
+      <x:c r="E20" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F20" s="46"/>
+      <x:c r="G20" s="46"/>
+      <x:c r="H20" s="46"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="46" t="str">
+        <x:v>1.3 µH</x:v>
+      </x:c>
+      <x:c r="B21" s="46" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C21" s="46"/>
+      <x:c r="D21" s="47" t="str">
+        <x:v>390 pF</x:v>
+      </x:c>
+      <x:c r="E21" s="46" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F21" s="46"/>
+      <x:c r="G21" s="46"/>
+      <x:c r="H21" s="46"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="46" t="str">
+        <x:v>1.69 µH</x:v>
+      </x:c>
+      <x:c r="B22" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C22" s="46"/>
+      <x:c r="D22" s="47" t="str">
+        <x:v>470 pF</x:v>
+      </x:c>
+      <x:c r="E22" s="46" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="F4" s="38"/>
-      <x:c r="G4" s="38"/>
-      <x:c r="H4" s="38"/>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="38" t="str">
-        <x:v>332 nH</x:v>
-      </x:c>
-      <x:c r="B5" s="38" t="n">
+      <x:c r="F22" s="46"/>
+      <x:c r="G22" s="46"/>
+      <x:c r="H22" s="46"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="46" t="str">
+        <x:v>1.78 µH</x:v>
+      </x:c>
+      <x:c r="B23" s="46" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C5" s="38"/>
-      <x:c r="D5" s="39" t="str">
-        <x:v>20 pF</x:v>
-      </x:c>
-      <x:c r="E5" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F5" s="38"/>
-      <x:c r="G5" s="38"/>
-      <x:c r="H5" s="38"/>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="38" t="str">
-        <x:v>357 nH</x:v>
-      </x:c>
-      <x:c r="B6" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C6" s="38"/>
-      <x:c r="D6" s="39" t="str">
-        <x:v>43 pF</x:v>
-      </x:c>
-      <x:c r="E6" s="38" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="F6" s="38"/>
-      <x:c r="G6" s="38"/>
-      <x:c r="H6" s="38"/>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="38" t="str">
-        <x:v>374 nH</x:v>
-      </x:c>
-      <x:c r="B7" s="38" t="n">
+      <x:c r="C23" s="46"/>
+      <x:c r="D23" s="47" t="str">
+        <x:v>511 pF</x:v>
+      </x:c>
+      <x:c r="E23" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F23" s="46"/>
+      <x:c r="G23" s="46"/>
+      <x:c r="H23" s="46"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="46" t="str">
+        <x:v>2.49 µH</x:v>
+      </x:c>
+      <x:c r="B24" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C24" s="46"/>
+      <x:c r="D24" s="47" t="str">
+        <x:v>560 pF</x:v>
+      </x:c>
+      <x:c r="E24" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F24" s="46"/>
+      <x:c r="G24" s="46"/>
+      <x:c r="H24" s="46"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="46" t="str">
+        <x:v>2.61 µH</x:v>
+      </x:c>
+      <x:c r="B25" s="46" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C7" s="38"/>
-      <x:c r="D7" s="39" t="str">
-        <x:v>51 pF</x:v>
-      </x:c>
-      <x:c r="E7" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F7" s="38"/>
-      <x:c r="G7" s="38"/>
-      <x:c r="H7" s="38"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="38" t="str">
-        <x:v>422 nH</x:v>
-      </x:c>
-      <x:c r="B8" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C8" s="38"/>
-      <x:c r="D8" s="39" t="str">
-        <x:v>75 pF</x:v>
-      </x:c>
-      <x:c r="E8" s="38" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="F8" s="38"/>
-      <x:c r="G8" s="38"/>
-      <x:c r="H8" s="38"/>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="38" t="str">
-        <x:v>442 nH</x:v>
-      </x:c>
-      <x:c r="B9" s="38" t="n">
+      <x:c r="C25" s="46"/>
+      <x:c r="D25" s="47" t="str">
+        <x:v>680 pF</x:v>
+      </x:c>
+      <x:c r="E25" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F25" s="46"/>
+      <x:c r="G25" s="46"/>
+      <x:c r="H25" s="46"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="46" t="str">
+        <x:v>4.87 µH</x:v>
+      </x:c>
+      <x:c r="B26" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C26" s="46"/>
+      <x:c r="D26" s="47" t="str">
+        <x:v>681 pF</x:v>
+      </x:c>
+      <x:c r="E26" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F26" s="46"/>
+      <x:c r="G26" s="46"/>
+      <x:c r="H26" s="46"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="46" t="str">
+        <x:v>5.11 µH</x:v>
+      </x:c>
+      <x:c r="B27" s="46" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C9" s="38"/>
-      <x:c r="D9" s="39" t="str">
-        <x:v>100 pF</x:v>
-      </x:c>
-      <x:c r="E9" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F9" s="38"/>
-      <x:c r="G9" s="38"/>
-      <x:c r="H9" s="38"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="38" t="str">
-        <x:v>487 nH</x:v>
-      </x:c>
-      <x:c r="B10" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C10" s="38"/>
-      <x:c r="D10" s="39" t="str">
-        <x:v>110 pF</x:v>
-      </x:c>
-      <x:c r="E10" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F10" s="38"/>
-      <x:c r="G10" s="38"/>
-      <x:c r="H10" s="38"/>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="38" t="str">
-        <x:v>511 nH</x:v>
-      </x:c>
-      <x:c r="B11" s="38" t="n">
+      <x:c r="C27" s="46"/>
+      <x:c r="D27" s="47" t="str">
+        <x:v>732 pF</x:v>
+      </x:c>
+      <x:c r="E27" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F27" s="46"/>
+      <x:c r="G27" s="46"/>
+      <x:c r="H27" s="46"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="46" t="str">
+        <x:v>18.7 µH</x:v>
+      </x:c>
+      <x:c r="B28" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C28" s="46"/>
+      <x:c r="D28" s="47" t="str">
+        <x:v>820 pF</x:v>
+      </x:c>
+      <x:c r="E28" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F28" s="46"/>
+      <x:c r="G28" s="46"/>
+      <x:c r="H28" s="46"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="46" t="str">
+        <x:v>19.6 µH</x:v>
+      </x:c>
+      <x:c r="B29" s="46" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C11" s="38"/>
-      <x:c r="D11" s="39" t="str">
-        <x:v>130 pF</x:v>
-      </x:c>
-      <x:c r="E11" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F11" s="38"/>
-      <x:c r="G11" s="38"/>
-      <x:c r="H11" s="38"/>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="38" t="str">
-        <x:v>634 nH</x:v>
-      </x:c>
-      <x:c r="B12" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C12" s="38"/>
-      <x:c r="D12" s="39" t="str">
-        <x:v>180 pF</x:v>
-      </x:c>
-      <x:c r="E12" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F12" s="38"/>
-      <x:c r="G12" s="38"/>
-      <x:c r="H12" s="38"/>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="38" t="str">
-        <x:v>649 nH</x:v>
-      </x:c>
-      <x:c r="B13" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C13" s="38"/>
-      <x:c r="D13" s="39" t="str">
-        <x:v>200 pF</x:v>
-      </x:c>
-      <x:c r="E13" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F13" s="38"/>
-      <x:c r="G13" s="38"/>
-      <x:c r="H13" s="38"/>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="38" t="str">
-        <x:v>665 nH</x:v>
-      </x:c>
-      <x:c r="B14" s="38" t="n">
+      <x:c r="C29" s="46"/>
+      <x:c r="D29" s="47" t="str">
+        <x:v>910 pF</x:v>
+      </x:c>
+      <x:c r="E29" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F29" s="46"/>
+      <x:c r="G29" s="46"/>
+      <x:c r="H29" s="46"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="46" t="str">
+        <x:v>64.9 µH</x:v>
+      </x:c>
+      <x:c r="B30" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C30" s="46"/>
+      <x:c r="D30" s="47" t="str">
+        <x:v>976 pF</x:v>
+      </x:c>
+      <x:c r="E30" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F30" s="46"/>
+      <x:c r="G30" s="46"/>
+      <x:c r="H30" s="46"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="46" t="str">
+        <x:v>68.1 µH</x:v>
+      </x:c>
+      <x:c r="B31" s="46" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C14" s="38"/>
-      <x:c r="D14" s="39" t="str">
-        <x:v>243 pF</x:v>
-      </x:c>
-      <x:c r="E14" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F14" s="38"/>
-      <x:c r="G14" s="38"/>
-      <x:c r="H14" s="38"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="38" t="str">
-        <x:v>681 nH</x:v>
-      </x:c>
-      <x:c r="B15" s="38" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C15" s="38"/>
-      <x:c r="D15" s="39" t="str">
-        <x:v>270 pF</x:v>
-      </x:c>
-      <x:c r="E15" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F15" s="38"/>
-      <x:c r="G15" s="38"/>
-      <x:c r="H15" s="38"/>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="38" t="str">
-        <x:v>866 nH</x:v>
-      </x:c>
-      <x:c r="B16" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C16" s="38"/>
-      <x:c r="D16" s="39" t="str">
-        <x:v>324 pF</x:v>
-      </x:c>
-      <x:c r="E16" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F16" s="38"/>
-      <x:c r="G16" s="38"/>
-      <x:c r="H16" s="38"/>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="38" t="str">
-        <x:v>909 nH</x:v>
-      </x:c>
-      <x:c r="B17" s="38" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C17" s="38"/>
-      <x:c r="D17" s="39" t="str">
-        <x:v>348 pF</x:v>
-      </x:c>
-      <x:c r="E17" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F17" s="38"/>
-      <x:c r="G17" s="38"/>
-      <x:c r="H17" s="38"/>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="38" t="str">
-        <x:v>1.27 µH</x:v>
-      </x:c>
-      <x:c r="B18" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C18" s="38"/>
-      <x:c r="D18" s="39" t="str">
-        <x:v>360 pF</x:v>
-      </x:c>
-      <x:c r="E18" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F18" s="38"/>
-      <x:c r="G18" s="38"/>
-      <x:c r="H18" s="38"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="38" t="str">
-        <x:v>1.3 µH</x:v>
-      </x:c>
-      <x:c r="B19" s="38" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C19" s="38"/>
-      <x:c r="D19" s="39" t="str">
-        <x:v>390 pF</x:v>
-      </x:c>
-      <x:c r="E19" s="38" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="F19" s="38"/>
-      <x:c r="G19" s="38"/>
-      <x:c r="H19" s="38"/>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="38" t="str">
-        <x:v>1.69 µH</x:v>
-      </x:c>
-      <x:c r="B20" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C20" s="38"/>
-      <x:c r="D20" s="39" t="str">
-        <x:v>470 pF</x:v>
-      </x:c>
-      <x:c r="E20" s="38" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="F20" s="38"/>
-      <x:c r="G20" s="38"/>
-      <x:c r="H20" s="38"/>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="38" t="str">
-        <x:v>1.78 µH</x:v>
-      </x:c>
-      <x:c r="B21" s="38" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C21" s="38"/>
-      <x:c r="D21" s="39" t="str">
-        <x:v>511 pF</x:v>
-      </x:c>
-      <x:c r="E21" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F21" s="38"/>
-      <x:c r="G21" s="38"/>
-      <x:c r="H21" s="38"/>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="38" t="str">
-        <x:v>2.49 µH</x:v>
-      </x:c>
-      <x:c r="B22" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C22" s="38"/>
-      <x:c r="D22" s="39" t="str">
-        <x:v>560 pF</x:v>
-      </x:c>
-      <x:c r="E22" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F22" s="38"/>
-      <x:c r="G22" s="38"/>
-      <x:c r="H22" s="38"/>
-    </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="38" t="str">
-        <x:v>2.61 µH</x:v>
-      </x:c>
-      <x:c r="B23" s="38" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C23" s="38"/>
-      <x:c r="D23" s="39" t="str">
-        <x:v>680 pF</x:v>
-      </x:c>
-      <x:c r="E23" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F23" s="38"/>
-      <x:c r="G23" s="38"/>
-      <x:c r="H23" s="38"/>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="38" t="str">
-        <x:v>4.87 µH</x:v>
-      </x:c>
-      <x:c r="B24" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C24" s="38"/>
-      <x:c r="D24" s="39" t="str">
-        <x:v>681 pF</x:v>
-      </x:c>
-      <x:c r="E24" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F24" s="38"/>
-      <x:c r="G24" s="38"/>
-      <x:c r="H24" s="38"/>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="38" t="str">
-        <x:v>5.11 µH</x:v>
-      </x:c>
-      <x:c r="B25" s="38" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C25" s="38"/>
-      <x:c r="D25" s="39" t="str">
-        <x:v>732 pF</x:v>
-      </x:c>
-      <x:c r="E25" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F25" s="38"/>
-      <x:c r="G25" s="38"/>
-      <x:c r="H25" s="38"/>
-    </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="38" t="str">
-        <x:v>18.7 µH</x:v>
-      </x:c>
-      <x:c r="B26" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C26" s="38"/>
-      <x:c r="D26" s="39" t="str">
-        <x:v>820 pF</x:v>
-      </x:c>
-      <x:c r="E26" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F26" s="38"/>
-      <x:c r="G26" s="38"/>
-      <x:c r="H26" s="38"/>
-    </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="38" t="str">
-        <x:v>19.6 µH</x:v>
-      </x:c>
-      <x:c r="B27" s="38" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C27" s="38"/>
-      <x:c r="D27" s="39" t="str">
-        <x:v>910 pF</x:v>
-      </x:c>
-      <x:c r="E27" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F27" s="38"/>
-      <x:c r="G27" s="38"/>
-      <x:c r="H27" s="38"/>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="38" t="str">
-        <x:v>64.9 µH</x:v>
-      </x:c>
-      <x:c r="B28" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C28" s="38"/>
-      <x:c r="D28" s="39" t="str">
-        <x:v>976 pF</x:v>
-      </x:c>
-      <x:c r="E28" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F28" s="38"/>
-      <x:c r="G28" s="38"/>
-      <x:c r="H28" s="38"/>
-    </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="38" t="str">
-        <x:v>68.1 µH</x:v>
-      </x:c>
-      <x:c r="B29" s="38" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C29" s="38"/>
-      <x:c r="D29" s="39" t="str">
+      <x:c r="C31" s="46"/>
+      <x:c r="D31" s="47" t="str">
         <x:v>1.3 nF</x:v>
       </x:c>
-      <x:c r="E29" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F29" s="38"/>
-      <x:c r="G29" s="38"/>
-      <x:c r="H29" s="38"/>
-    </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="38"/>
-      <x:c r="B30" s="38"/>
-      <x:c r="C30" s="38"/>
-      <x:c r="D30" s="39" t="str">
+      <x:c r="E31" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F31" s="46"/>
+      <x:c r="G31" s="46"/>
+      <x:c r="H31" s="46"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="46"/>
+      <x:c r="B32" s="46"/>
+      <x:c r="C32" s="46"/>
+      <x:c r="D32" s="47" t="str">
         <x:v>1.8 nF</x:v>
       </x:c>
-      <x:c r="E30" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F30" s="38"/>
-      <x:c r="G30" s="38"/>
-      <x:c r="H30" s="38"/>
-    </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="38"/>
-      <x:c r="B31" s="38"/>
-      <x:c r="C31" s="38"/>
-      <x:c r="D31" s="39" t="str">
+      <x:c r="E32" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F32" s="46"/>
+      <x:c r="G32" s="46"/>
+      <x:c r="H32" s="46"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="46"/>
+      <x:c r="B33" s="46"/>
+      <x:c r="C33" s="46"/>
+      <x:c r="D33" s="47" t="str">
         <x:v>1.91 nF</x:v>
       </x:c>
-      <x:c r="E31" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F31" s="38"/>
-      <x:c r="G31" s="38"/>
-      <x:c r="H31" s="38"/>
-    </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="38"/>
-      <x:c r="B32" s="38"/>
-      <x:c r="C32" s="38"/>
-      <x:c r="D32" s="39" t="str">
+      <x:c r="E33" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F33" s="46"/>
+      <x:c r="G33" s="46"/>
+      <x:c r="H33" s="46"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="46"/>
+      <x:c r="B34" s="46"/>
+      <x:c r="C34" s="46"/>
+      <x:c r="D34" s="47" t="str">
         <x:v>2.4 nF</x:v>
       </x:c>
-      <x:c r="E32" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F32" s="38"/>
-      <x:c r="G32" s="38"/>
-      <x:c r="H32" s="38"/>
-    </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="38"/>
-      <x:c r="B33" s="38"/>
-      <x:c r="C33" s="38"/>
-      <x:c r="D33" s="39" t="str">
+      <x:c r="E34" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F34" s="46"/>
+      <x:c r="G34" s="46"/>
+      <x:c r="H34" s="46"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="46"/>
+      <x:c r="B35" s="46"/>
+      <x:c r="C35" s="46"/>
+      <x:c r="D35" s="47" t="str">
         <x:v>2.7 nF</x:v>
       </x:c>
-      <x:c r="E33" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F33" s="38"/>
-      <x:c r="G33" s="38"/>
-      <x:c r="H33" s="38"/>
-    </x:row>
-    <x:row r="34">
-      <x:c r="A34" s="38"/>
-      <x:c r="B34" s="38"/>
-      <x:c r="C34" s="38"/>
-      <x:c r="D34" s="39" t="str">
+      <x:c r="E35" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F35" s="46"/>
+      <x:c r="G35" s="46"/>
+      <x:c r="H35" s="46"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="46"/>
+      <x:c r="B36" s="46"/>
+      <x:c r="C36" s="46"/>
+      <x:c r="D36" s="47" t="str">
         <x:v>3.6 nF</x:v>
       </x:c>
-      <x:c r="E34" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F34" s="38"/>
-      <x:c r="G34" s="38"/>
-      <x:c r="H34" s="38"/>
-    </x:row>
-    <x:row r="35">
-      <x:c r="A35" s="38"/>
-      <x:c r="B35" s="38"/>
-      <x:c r="C35" s="38"/>
-      <x:c r="D35" s="39" t="str">
+      <x:c r="E36" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F36" s="46"/>
+      <x:c r="G36" s="46"/>
+      <x:c r="H36" s="46"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="46"/>
+      <x:c r="B37" s="46"/>
+      <x:c r="C37" s="46"/>
+      <x:c r="D37" s="47" t="str">
         <x:v>5.1 nF</x:v>
       </x:c>
-      <x:c r="E35" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F35" s="38"/>
-      <x:c r="G35" s="38"/>
-      <x:c r="H35" s="38"/>
-    </x:row>
-    <x:row r="36">
-      <x:c r="A36" s="38"/>
-      <x:c r="B36" s="38"/>
-      <x:c r="C36" s="38"/>
-      <x:c r="D36" s="39" t="str">
+      <x:c r="E37" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F37" s="46"/>
+      <x:c r="G37" s="46"/>
+      <x:c r="H37" s="46"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="46"/>
+      <x:c r="B38" s="46"/>
+      <x:c r="C38" s="46"/>
+      <x:c r="D38" s="47" t="str">
         <x:v>9.1 nF</x:v>
       </x:c>
-      <x:c r="E36" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F36" s="38"/>
-      <x:c r="G36" s="38"/>
-      <x:c r="H36" s="38"/>
-    </x:row>
-    <x:row r="37">
-      <x:c r="A37" s="38"/>
-      <x:c r="B37" s="38"/>
-      <x:c r="C37" s="38"/>
-      <x:c r="D37" s="39" t="str">
+      <x:c r="E38" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F38" s="46"/>
+      <x:c r="G38" s="46"/>
+      <x:c r="H38" s="46"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="46"/>
+      <x:c r="B39" s="46"/>
+      <x:c r="C39" s="46"/>
+      <x:c r="D39" s="47" t="str">
         <x:v>14.3 nF</x:v>
       </x:c>
-      <x:c r="E37" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F37" s="38"/>
-      <x:c r="G37" s="38"/>
-      <x:c r="H37" s="38"/>
-    </x:row>
-    <x:row r="38">
-      <x:c r="A38" s="38"/>
-      <x:c r="B38" s="38"/>
-      <x:c r="C38" s="38"/>
-      <x:c r="D38" s="39" t="str">
+      <x:c r="E39" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F39" s="46"/>
+      <x:c r="G39" s="46"/>
+      <x:c r="H39" s="46"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="46"/>
+      <x:c r="B40" s="46"/>
+      <x:c r="C40" s="46"/>
+      <x:c r="D40" s="47" t="str">
         <x:v>20 nF</x:v>
       </x:c>
-      <x:c r="E38" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F38" s="38"/>
-      <x:c r="G38" s="38"/>
-      <x:c r="H38" s="38"/>
-    </x:row>
-    <x:row r="39">
-      <x:c r="A39" s="38"/>
-      <x:c r="B39" s="38"/>
-      <x:c r="C39" s="38"/>
-      <x:c r="D39" s="39" t="str">
+      <x:c r="E40" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F40" s="46"/>
+      <x:c r="G40" s="46"/>
+      <x:c r="H40" s="46"/>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="46"/>
+      <x:c r="B41" s="46"/>
+      <x:c r="C41" s="46"/>
+      <x:c r="D41" s="47" t="str">
         <x:v>47 nF</x:v>
       </x:c>
-      <x:c r="E39" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F39" s="38"/>
-      <x:c r="G39" s="38"/>
-      <x:c r="H39" s="38"/>
-    </x:row>
-    <x:row r="40">
-      <x:c r="A40" s="38"/>
-      <x:c r="B40" s="38"/>
-      <x:c r="C40" s="38"/>
-      <x:c r="D40" s="39" t="str">
+      <x:c r="E41" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F41" s="46"/>
+      <x:c r="G41" s="46"/>
+      <x:c r="H41" s="46"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="46"/>
+      <x:c r="B42" s="46"/>
+      <x:c r="C42" s="46"/>
+      <x:c r="D42" s="47" t="str">
         <x:v>62 nF</x:v>
       </x:c>
-      <x:c r="E40" s="38" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F40" s="38"/>
-      <x:c r="G40" s="38"/>
-      <x:c r="H40" s="38"/>
+      <x:c r="E42" s="46" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F42" s="46"/>
+      <x:c r="G42" s="46"/>
+      <x:c r="H42" s="46"/>
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="R1eb004ae682e40ce"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="R493619d0d9b641fe"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="Re4c440f861104a34"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="Rd720bed0cdfb4f6f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="R8c65e8b62bdf4eac"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="Ra5df5a84f5b84c55"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="R18c986dd8dfc41fa"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="R84d4ce0a6fc54478"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="Rd77403ecc01d4650"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="R1465ecb0759349c0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="R771b9cb5922c412f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="Ra3a99d65ba9248d0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="Re546da032ffc407c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="R77699e0cb5444489"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="R062364d147094f9c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="R8b20246c24ac42fe"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="R5697ba28e3cc4f98"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="Rf9d6ff43d0a34815"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="Rb6bd2a4f06dc48c3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="R2dc2bb324bac4c65"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="R3a18907c71dd4a3e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="R02e95f9ba31242c0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="R38a25c21243e42bb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="Ra02a5489a70d46ac"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="R85f6bf73f1794f2a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="Rf384cec83e504038"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="R53a4503f6ad64675"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="R7c13fe58f4cc4145"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="Re1e4a86e48a54f53"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="Rc995215a202f45c2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="R8784ab9ed9c4449a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="R87fa906a53e94b34"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="R7307d46710c24657"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="R4d455a1117044c53"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="R1b68f8fdd82f42b5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="R3602078c4dfc4021"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="R1ed77d7766a34f82"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="Ref0d28439bdf4bdd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="Re90a7b509b4e48b2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="Rd93fe4efbc7d4e70"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="R472be919b7604903"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="Re6baa2a43b454d8b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="R01a2456202194f32"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="Raecdb98118574449"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="R374ff97eeb3e4bbe"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="R82ee29cd18064ada"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="R857cebc7edd44be0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="Rf09a75edfa6440c0"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>